<commit_message>
Rename update_financials.js to report.js, add 1099 support, improve vendor validation
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="76">
   <si>
     <t>Category</t>
   </si>
@@ -66,54 +66,54 @@
     <t>Starbucks</t>
   </si>
   <si>
+    <t>Rent</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
+  <si>
+    <t>Expense</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Checking Account</t>
+  </si>
+  <si>
+    <t>Bank</t>
+  </si>
+  <si>
+    <t>Asset</t>
+  </si>
+  <si>
+    <t>Balance Sheet</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
     <t>Bank Transactions</t>
   </si>
   <si>
-    <t>Bank</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
-    <t>Rent</t>
-  </si>
-  <si>
-    <t>Office</t>
-  </si>
-  <si>
-    <t>Expense</t>
-  </si>
-  <si>
-    <t>Amazon</t>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>Liability</t>
   </si>
   <si>
     <t>Credit Card Transactions</t>
   </si>
   <si>
-    <t>CC</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Checking Account</t>
-  </si>
-  <si>
-    <t>Asset</t>
-  </si>
-  <si>
-    <t>Balance Sheet</t>
-  </si>
-  <si>
-    <t>AWS</t>
-  </si>
-  <si>
-    <t>Credit Card</t>
-  </si>
-  <si>
-    <t>Liability</t>
-  </si>
-  <si>
     <t>AX CC</t>
   </si>
   <si>
@@ -156,27 +156,24 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>d30caf8818b4bcec55d88484ee588c128f9dcf14</t>
+    <t>08e57897eb9bef642112c259c3a4bfb2a0f1dab6</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>12/30/2025, 11:11:02 AM</t>
+    <t>1/19/2026, 8:01:56 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 12/30/2025, 11:11:02 AM</t>
+    <t>Import at 1/19/2026, 8:01:56 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
-  </si>
-  <si>
-    <t>Import at 12/30/2025, 11:11:03 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -702,7 +699,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -718,77 +715,77 @@
       <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="I2" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="J2" t="s">
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="K2" t="s">
+      <c r="C3" t="s">
         <v>18</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
       </c>
       <c r="F3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
         <v>22</v>
       </c>
-      <c r="I3" t="s">
+      <c r="D4" t="s">
         <v>23</v>
       </c>
-      <c r="J3" t="s">
+      <c r="F4" t="s">
         <v>24</v>
       </c>
-      <c r="K3" t="s">
+      <c r="I4" t="s">
         <v>25</v>
       </c>
-      <c r="L3">
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="F4" t="s">
+      <c r="C5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
-        <v>28</v>
+      <c r="L5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -796,13 +793,13 @@
         <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -813,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
         <v>14</v>
@@ -821,13 +818,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
         <v>14</v>
@@ -855,7 +852,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -863,7 +860,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -877,7 +874,7 @@
         <v>35</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -886,16 +883,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -903,7 +900,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -915,7 +912,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -932,19 +929,19 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C5">
         <v>-1500</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -961,7 +958,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -973,7 +970,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -990,22 +987,22 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
         <v>68</v>
-      </c>
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s">
-        <v>69</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1016,7 +1013,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1076,7 +1073,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1084,7 +1081,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1095,13 +1092,13 @@
         <v>34</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1110,22 +1107,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1148,7 +1145,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1174,19 +1171,19 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D5">
         <v>120</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1212,19 +1209,19 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D6">
         <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1302,7 +1299,7 @@
         <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D2">
         <v>1000</v>
@@ -1319,7 +1316,7 @@
         <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D3">
         <v>50</v>
@@ -1403,10 +1400,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Report: Add missing vendors list and 1099 details
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -156,19 +156,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>08e57897eb9bef642112c259c3a4bfb2a0f1dab6</t>
+    <t>0342a2e046709e8c9bdadb7cdfe32b6cf23cc4fe</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 8:01:56 AM</t>
+    <t>1/19/2026, 8:13:16 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 8:01:56 AM</t>
+    <t>Import at 1/19/2026, 8:13:17 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Debug: Enhance 1099 visibility (threshold skipping, detection logs)
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="77">
   <si>
     <t>Category</t>
   </si>
@@ -156,24 +156,27 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>0342a2e046709e8c9bdadb7cdfe32b6cf23cc4fe</t>
+    <t>6dd29c410f440e426d6c2095a338733de5f1af13</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 8:13:16 AM</t>
+    <t>1/19/2026, 8:31:55 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 8:13:17 AM</t>
+    <t>Import at 1/19/2026, 8:31:55 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
+  </si>
+  <si>
+    <t>Import at 1/19/2026, 8:31:56 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -852,7 +855,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -860,7 +863,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -874,7 +877,7 @@
         <v>35</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -883,16 +886,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -900,7 +903,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -912,7 +915,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -929,7 +932,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -941,7 +944,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -958,7 +961,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -970,7 +973,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -987,13 +990,13 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E7" t="s">
         <v>4</v>
@@ -1002,7 +1005,7 @@
         <v>4</v>
       </c>
       <c r="G7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1013,7 +1016,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1073,7 +1076,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1081,7 +1084,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1092,13 +1095,13 @@
         <v>34</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1107,22 +1110,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1145,7 +1148,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1183,7 +1186,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1221,7 +1224,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1400,10 +1403,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor: 1099 polarity/thresholds and JS rules
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -156,19 +156,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>6dd29c410f440e426d6c2095a338733de5f1af13</t>
+    <t>775bfaaa976a6bc6b5d4981e5af194cf62fbd7bc</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 8:31:55 AM</t>
+    <t>1/19/2026, 8:37:32 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 8:31:55 AM</t>
+    <t>Import at 1/19/2026, 8:37:32 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
@@ -176,7 +176,7 @@
 Target Sheet: Bank Transactions</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 8:31:56 AM</t>
+    <t>Import at 1/19/2026, 8:37:33 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Feat: 1099 CSV gen, external vendor file, split 1099 setup cols
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="76">
   <si>
     <t>Category</t>
   </si>
@@ -156,27 +156,24 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>775bfaaa976a6bc6b5d4981e5af194cf62fbd7bc</t>
+    <t>75efa489171bca23b18d980eeadde070c5aec29d</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 8:37:32 AM</t>
+    <t>1/19/2026, 8:58:34 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 8:37:32 AM</t>
+    <t>Import at 1/19/2026, 8:58:34 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
-  </si>
-  <si>
-    <t>Import at 1/19/2026, 8:37:33 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -855,7 +852,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -863,7 +860,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -877,7 +874,7 @@
         <v>35</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -886,16 +883,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -903,7 +900,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -915,7 +912,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -932,7 +929,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -944,7 +941,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -961,7 +958,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -973,7 +970,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -990,22 +987,22 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
         <v>68</v>
-      </c>
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s">
-        <v>69</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1016,7 +1013,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1076,7 +1073,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1084,7 +1081,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1095,13 +1092,13 @@
         <v>34</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1110,22 +1107,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1148,7 +1145,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1186,7 +1183,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1224,7 +1221,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1403,10 +1400,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor: Silent 1099 report, enhanced Vendor report columns
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
   <si>
     <t>Category</t>
   </si>
@@ -120,6 +120,15 @@
     <t>Travel</t>
   </si>
   <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>Contractor 1099</t>
+  </si>
+  <si>
+    <t>NEC</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -156,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>75efa489171bca23b18d980eeadde070c5aec29d</t>
+    <t>c10e2ab68e7ca94c29d17fe0749eb08c6a361071</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 8:58:34 AM</t>
+    <t>1/19/2026, 9:04:53 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 8:58:34 AM</t>
+    <t>Import at 1/19/2026, 9:04:53 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
@@ -176,6 +185,9 @@
 Target Sheet: Bank Transactions</t>
   </si>
   <si>
+    <t>Import at 1/19/2026, 9:04:54 AM</t>
+  </si>
+  <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
 Input: tests/example_cc.csv
 Target Sheet: Credit Card Transactions</t>
@@ -230,6 +242,9 @@
   </si>
   <si>
     <t>Uncategorized Expense</t>
+  </si>
+  <si>
+    <t>Major Contract Work</t>
   </si>
   <si>
     <t>Member</t>
@@ -647,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="25" customWidth="1"/>
@@ -818,7 +833,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
@@ -828,6 +843,42 @@
       </c>
       <c r="D8" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -838,7 +889,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -852,7 +903,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -860,7 +911,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -868,13 +919,13 @@
     </row>
     <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -883,16 +934,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -900,7 +951,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -912,7 +963,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -929,7 +980,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -941,7 +992,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -958,7 +1009,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -970,7 +1021,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -987,13 +1038,13 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E7" t="s">
         <v>4</v>
@@ -1002,7 +1053,7 @@
         <v>4</v>
       </c>
       <c r="G7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1013,7 +1064,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1031,6 +1082,32 @@
         <v>4</v>
       </c>
       <c r="H8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>45684</v>
+      </c>
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9">
+        <v>-737.5</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G9" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1073,7 +1150,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1081,7 +1158,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1089,16 +1166,16 @@
     </row>
     <row r="3" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1107,22 +1184,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1145,7 +1222,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1183,7 +1260,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1221,7 +1298,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1273,22 +1350,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1296,7 +1373,7 @@
         <v>45658</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C2" t="s">
         <v>20</v>
@@ -1313,7 +1390,7 @@
         <v>45677</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
         <v>17</v>
@@ -1352,39 +1429,39 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
@@ -1392,18 +1469,18 @@
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Normalized header lookup for 1099 and Payer Info
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="80">
   <si>
     <t>Category</t>
   </si>
@@ -165,27 +165,24 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>c10e2ab68e7ca94c29d17fe0749eb08c6a361071</t>
+    <t>6020f1050e3f809f7efa38bb0fe90f03f6ddaea7</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 9:04:53 AM</t>
+    <t>1/19/2026, 9:07:14 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 9:04:53 AM</t>
+    <t>Import at 1/19/2026, 9:07:15 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
-  </si>
-  <si>
-    <t>Import at 1/19/2026, 9:04:54 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -903,7 +900,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -911,7 +908,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -925,7 +922,7 @@
         <v>38</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -934,16 +931,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -951,7 +948,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -963,7 +960,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -980,7 +977,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -992,7 +989,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -1009,7 +1006,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -1021,7 +1018,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -1038,22 +1035,22 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
         <v>71</v>
-      </c>
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s">
-        <v>72</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1064,7 +1061,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1090,7 +1087,7 @@
         <v>45684</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9">
         <v>-737.5</v>
@@ -1150,7 +1147,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1158,7 +1155,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1169,13 +1166,13 @@
         <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1184,22 +1181,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1222,7 +1219,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1260,7 +1257,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1298,7 +1295,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1477,10 +1474,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Crash in 1099 logic and missing vendor columns
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
   <si>
     <t>Category</t>
   </si>
@@ -165,24 +165,27 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>6020f1050e3f809f7efa38bb0fe90f03f6ddaea7</t>
+    <t>1f1a8641d5e9d2443eb3deee253c14a96601b746</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 9:07:14 AM</t>
+    <t>1/19/2026, 9:11:31 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 9:07:15 AM</t>
+    <t>Import at 1/19/2026, 9:11:31 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
+  </si>
+  <si>
+    <t>Import at 1/19/2026, 9:11:32 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -900,7 +903,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -908,7 +911,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -922,7 +925,7 @@
         <v>38</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -931,16 +934,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -948,7 +951,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -960,7 +963,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -977,7 +980,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -989,7 +992,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -1006,7 +1009,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -1018,7 +1021,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -1035,13 +1038,13 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E7" t="s">
         <v>4</v>
@@ -1050,7 +1053,7 @@
         <v>4</v>
       </c>
       <c r="G7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1061,7 +1064,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1087,7 +1090,7 @@
         <v>45684</v>
       </c>
       <c r="B9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C9">
         <v>-737.5</v>
@@ -1147,7 +1150,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1155,7 +1158,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1166,13 +1169,13 @@
         <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1181,22 +1184,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1219,7 +1222,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1257,7 +1260,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1295,7 +1298,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1474,10 +1477,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Polarity corrected to Positive Magnitude for Expenses
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="80">
   <si>
     <t>Category</t>
   </si>
@@ -165,27 +165,24 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>1f1a8641d5e9d2443eb3deee253c14a96601b746</t>
+    <t>292b52095847cc5d06dbf4123f7d694df0b4e379</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 9:11:31 AM</t>
+    <t>1/19/2026, 9:30:39 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 9:11:31 AM</t>
+    <t>Import at 1/19/2026, 9:30:40 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
-  </si>
-  <si>
-    <t>Import at 1/19/2026, 9:11:32 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -903,7 +900,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -911,7 +908,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -925,7 +922,7 @@
         <v>38</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -934,16 +931,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -951,7 +948,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -963,7 +960,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -980,7 +977,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -992,7 +989,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -1009,7 +1006,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -1021,7 +1018,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -1038,22 +1035,22 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
         <v>71</v>
-      </c>
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s">
-        <v>72</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1064,7 +1061,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1090,7 +1087,7 @@
         <v>45684</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9">
         <v>-737.5</v>
@@ -1150,7 +1147,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1158,7 +1155,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1169,13 +1166,13 @@
         <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1184,22 +1181,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1222,7 +1219,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1260,7 +1257,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1298,7 +1295,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1477,10 +1474,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Vendor Report Polarity (Positive = Spending) and 1099 Output
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -165,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>292b52095847cc5d06dbf4123f7d694df0b4e379</t>
+    <t>34a0cae8d7702e312eb7c8492a36f9ea7c06db20</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 9:30:39 AM</t>
+    <t>1/19/2026, 9:35:08 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 9:30:40 AM</t>
+    <t>Import at 1/19/2026, 9:35:09 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Fix: Required column now shows YES for legacy 1099 vendors
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -165,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>34a0cae8d7702e312eb7c8492a36f9ea7c06db20</t>
+    <t>d6de0d8f68cacef702e70e9ad7b92b90be714b41</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 9:35:08 AM</t>
+    <t>1/19/2026, 2:18:28 PM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 9:35:09 AM</t>
+    <t>Import at 1/19/2026, 2:18:29 PM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Fix: Required column now respects thresholds + compliance test
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -165,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>d6de0d8f68cacef702e70e9ad7b92b90be714b41</t>
+    <t>2abc7ab878d967f486d878f4c519529c8d002d9e</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 2:18:28 PM</t>
+    <t>1/19/2026, 2:21:02 PM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 2:18:29 PM</t>
+    <t>Import at 1/19/2026, 2:21:03 PM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Fix: Add subcategory validation to checker
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
   <si>
     <t>Category</t>
   </si>
@@ -165,24 +165,27 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>2abc7ab878d967f486d878f4c519529c8d002d9e</t>
+    <t>5d1ad0cd53106a74e85b2f0d396f3f1b79507dc0</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/19/2026, 2:21:02 PM</t>
+    <t>1/20/2026, 9:24:20 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/19/2026, 2:21:03 PM</t>
+    <t>Import at 1/20/2026, 9:24:20 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
+  </si>
+  <si>
+    <t>Import at 1/20/2026, 9:24:21 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -900,7 +903,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -908,7 +911,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -922,7 +925,7 @@
         <v>38</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -931,16 +934,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -948,7 +951,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -960,7 +963,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -977,7 +980,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -989,7 +992,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -1006,7 +1009,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -1018,7 +1021,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -1035,13 +1038,13 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E7" t="s">
         <v>4</v>
@@ -1050,7 +1053,7 @@
         <v>4</v>
       </c>
       <c r="G7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1061,7 +1064,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1087,7 +1090,7 @@
         <v>45684</v>
       </c>
       <c r="B9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C9">
         <v>-737.5</v>
@@ -1147,7 +1150,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1155,7 +1158,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1166,13 +1169,13 @@
         <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1181,22 +1184,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1219,7 +1222,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1257,7 +1260,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1295,7 +1298,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1474,10 +1477,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Robustness: Add Ledger subcat validation, date/NaN checks
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="80">
   <si>
     <t>Category</t>
   </si>
@@ -165,27 +165,24 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>5d1ad0cd53106a74e85b2f0d396f3f1b79507dc0</t>
+    <t>51e02987e93ff90ead43ba052e4940cc67038893</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/20/2026, 9:24:20 AM</t>
+    <t>1/20/2026, 9:27:48 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/20/2026, 9:24:20 AM</t>
+    <t>Import at 1/20/2026, 9:27:48 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear
 Input: tests/example_bank.csv
 Target Sheet: Bank Transactions</t>
-  </si>
-  <si>
-    <t>Import at 1/20/2026, 9:24:21 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_cc.csv cc Test_Accounting.xlsx --clear
@@ -903,7 +900,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C1" s="3">
         <f>SUM(C4:C10000)</f>
@@ -911,7 +908,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C2" s="4">
         <f>SUBTOTAL(109, C4:C10000)</f>
@@ -925,7 +922,7 @@
         <v>38</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>0</v>
@@ -934,16 +931,16 @@
         <v>1</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -951,7 +948,7 @@
         <v>45658</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C4">
         <v>5000</v>
@@ -963,7 +960,7 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G4" t="s">
         <v>4</v>
@@ -980,7 +977,7 @@
         <v>45662</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5">
         <v>-1500</v>
@@ -992,7 +989,7 @@
         <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G5" t="s">
         <v>4</v>
@@ -1009,7 +1006,7 @@
         <v>45667</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6">
         <v>2500</v>
@@ -1021,7 +1018,7 @@
         <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
         <v>4</v>
@@ -1038,22 +1035,22 @@
         <v>45682</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C7">
         <v>100</v>
       </c>
       <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" t="s">
         <v>71</v>
-      </c>
-      <c r="E7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" t="s">
-        <v>72</v>
       </c>
       <c r="H7" t="s">
         <v>4</v>
@@ -1064,7 +1061,7 @@
         <v>45683</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8">
         <v>50</v>
@@ -1090,7 +1087,7 @@
         <v>45684</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C9">
         <v>-737.5</v>
@@ -1150,7 +1147,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D1" s="3">
         <f>SUM(D4:D10000)</f>
@@ -1158,7 +1155,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" s="4">
         <f>SUBTOTAL(109, D4:D10000)</f>
@@ -1169,13 +1166,13 @@
         <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>0</v>
@@ -1184,22 +1181,22 @@
         <v>1</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1222,7 +1219,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H4" t="s">
         <v>4</v>
@@ -1260,7 +1257,7 @@
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H5" t="s">
         <v>4</v>
@@ -1298,7 +1295,7 @@
         <v>4</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H6" t="s">
         <v>4</v>
@@ -1477,10 +1474,10 @@
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feature: Add --bs-sub flag for Balance Sheet subcategories
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -165,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>51e02987e93ff90ead43ba052e4940cc67038893</t>
+    <t>c14999f54567b78bfc17fd3e585ddcfdd2cb4a1d</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/20/2026, 9:27:48 AM</t>
+    <t>1/20/2026, 9:32:45 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/20/2026, 9:27:48 AM</t>
+    <t>Import at 1/20/2026, 9:32:46 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Fix: Only warn on Report type conflicts, not valid subcategory definitions
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -165,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>c14999f54567b78bfc17fd3e585ddcfdd2cb4a1d</t>
+    <t>3b3417b977c48563bcff2c1535b48f17084d451c</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/20/2026, 9:32:45 AM</t>
+    <t>1/20/2026, 10:13:41 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/20/2026, 9:32:46 AM</t>
+    <t>Import at 1/20/2026, 10:13:42 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Feature: Detect vendors/customers used in both P&L and BS
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -165,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>3b3417b977c48563bcff2c1535b48f17084d451c</t>
+    <t>925f4f97e763f30c512aaaa304adccecfaed1e5c</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/20/2026, 10:13:41 AM</t>
+    <t>1/20/2026, 10:25:45 AM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/20/2026, 10:13:42 AM</t>
+    <t>Import at 1/20/2026, 10:25:46 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>

<commit_message>
Fix: Apply vendor/customer report tracking to Ledger transactions
</commit_message>
<xml_diff>
--- a/tests/Full_Accounting_Test_Case.xlsx
+++ b/tests/Full_Accounting_Test_Case.xlsx
@@ -165,19 +165,19 @@
     <t>Git SHA</t>
   </si>
   <si>
-    <t>925f4f97e763f30c512aaaa304adccecfaed1e5c</t>
+    <t>5bab65fd3b3bfd11deb9b900711e268940bb6749</t>
   </si>
   <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>1/20/2026, 10:25:45 AM</t>
+    <t>1/20/2026, 2:48:12 PM</t>
   </si>
   <si>
     <t>--- Import History ---</t>
   </si>
   <si>
-    <t>Import at 1/20/2026, 10:25:46 AM</t>
+    <t>Import at 1/20/2026, 2:48:12 PM</t>
   </si>
   <si>
     <t xml:space="preserve">Command: node load_transactions.js tests/example_bank.csv bank Test_Accounting.xlsx --clear

</xml_diff>